<commit_message>
fix: normalizar estudios/genero pandape y corregir cedulas en plantilla
- pandape_views.py: _norm_estudios extrae nivel de educacion del formato
  institucion . nivel y trunca a 60 chars (max_length); el 78% de registros
  excedia el limite causando DataError. _norm_genero mapea Hombre/Mujer a
  MASCULINO/FEMENINO/OTRO
- Plantilla xlsx: reemplazar cedulas y correos reales en ejemplos por valores
  ficticios (1111100001/2/3) para evitar colision con BD real que activaba
  el check nombre_incoherente y reportaba error en fila 4

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/Plantilla_Carga_Trazabilidad_Euro.xlsx
+++ b/recursos/Plantilla_Carga_Trazabilidad_Euro.xlsx
@@ -684,7 +684,7 @@
     <row r="2" ht="43.95" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>1032455010</t>
+          <t>1111100001</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>carlosarboleda@gmail.com</t>
+          <t>ejemplo1@ejemplo.com</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr">
@@ -791,7 +791,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>1046953342</t>
+          <t>1111100002</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -837,7 +837,7 @@
       <c r="J3" s="5" t="n"/>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>abel.puerta@hotmail.com</t>
+          <t>ejemplo2@ejemplo.com</t>
         </is>
       </c>
       <c r="L3" s="5" t="inlineStr">
@@ -894,7 +894,7 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>1128443195</t>
+          <t>1111100003</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>jessica.rendon@gmail.com</t>
+          <t>ejemplo3@ejemplo.com</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">

</xml_diff>